<commit_message>
WG South east Asia sheet name
</commit_message>
<xml_diff>
--- a/data/2026_S_F_WG.xlsx
+++ b/data/2026_S_F_WG.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{50F96465-786E-4F9B-8F60-C3E903D67B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29129FC9-F80A-4C67-8817-41C99A5E6BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{355F51DA-C17A-4A57-BF4D-C39486966AED}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="South Asia" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>